<commit_message>
mergeo pequeño cambio pendiente
</commit_message>
<xml_diff>
--- a/Clase 5 - Markdown, loops y funciones/funciones y loops/bases/ipc_trimestral.xlsx
+++ b/Clase 5 - Markdown, loops y funciones/funciones y loops/bases/ipc_trimestral.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Guido\Trabajo\Repositorios de R\Cursos de R\Curso R_mercado de trabajo\curso_aset\Clase 5 - Markdown, loops y funciones\funciones y loops\bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Guido W\curso_aset\Clase 5 - Markdown, loops y funciones\funciones y loops\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62E3D70-1EBE-465D-8486-7919FD5B4E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AA1763-D1B1-47A3-8D27-0CF2A0F63BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="31">
   <si>
     <t>Período</t>
   </si>
@@ -132,10 +132,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -158,14 +171,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -459,10 +475,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E83"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F88"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -479,7 +495,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -497,7 +513,7 @@
         <v>2003T3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -515,7 +531,7 @@
         <v>2003T4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -533,7 +549,7 @@
         <v>2004T1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -551,7 +567,7 @@
         <v>2004T2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -569,7 +585,7 @@
         <v>2004T3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -587,7 +603,7 @@
         <v>2004T4</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -605,7 +621,7 @@
         <v>2005T1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -623,7 +639,7 @@
         <v>2005T2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -641,7 +657,7 @@
         <v>2005T3</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -659,7 +675,7 @@
         <v>2005T4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -677,7 +693,7 @@
         <v>2006T1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -695,7 +711,7 @@
         <v>2006T2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -713,7 +729,7 @@
         <v>2006T3</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -731,7 +747,7 @@
         <v>2006T4</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -749,7 +765,7 @@
         <v>2007T1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -767,7 +783,7 @@
         <v>2007T2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -785,7 +801,7 @@
         <v>2007T3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -803,7 +819,7 @@
         <v>2007T4</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -821,7 +837,7 @@
         <v>2008T1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -839,7 +855,7 @@
         <v>2008T2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -857,7 +873,7 @@
         <v>2008T3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -875,7 +891,7 @@
         <v>2008T4</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -893,7 +909,7 @@
         <v>2009T1</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -911,7 +927,7 @@
         <v>2009T2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -929,7 +945,7 @@
         <v>2009T3</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -947,7 +963,7 @@
         <v>2009T4</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -965,7 +981,7 @@
         <v>2010T1</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -983,7 +999,7 @@
         <v>2010T2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1001,7 +1017,7 @@
         <v>2010T3</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -1019,7 +1035,7 @@
         <v>2010T4</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>16</v>
       </c>
@@ -1037,7 +1053,7 @@
         <v>2011T1</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>16</v>
       </c>
@@ -1055,7 +1071,7 @@
         <v>2011T2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>16</v>
       </c>
@@ -1073,7 +1089,7 @@
         <v>2011T3</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>16</v>
       </c>
@@ -1091,7 +1107,7 @@
         <v>2011T4</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -1109,7 +1125,7 @@
         <v>2012T1</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>17</v>
       </c>
@@ -1127,7 +1143,7 @@
         <v>2012T2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>17</v>
       </c>
@@ -1145,7 +1161,7 @@
         <v>2012T3</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>17</v>
       </c>
@@ -1163,7 +1179,7 @@
         <v>2012T4</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>18</v>
       </c>
@@ -1181,7 +1197,7 @@
         <v>2013T1</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>18</v>
       </c>
@@ -1199,7 +1215,7 @@
         <v>2013T2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>18</v>
       </c>
@@ -1217,7 +1233,7 @@
         <v>2013T3</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1235,7 +1251,7 @@
         <v>2013T4</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1253,7 +1269,7 @@
         <v>2014T1</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -1271,7 +1287,7 @@
         <v>2014T2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -1289,7 +1305,7 @@
         <v>2014T3</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -1307,7 +1323,7 @@
         <v>2014T4</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>20</v>
       </c>
@@ -1325,7 +1341,7 @@
         <v>2015T1</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>20</v>
       </c>
@@ -1343,7 +1359,7 @@
         <v>2015T2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>20</v>
       </c>
@@ -1361,7 +1377,7 @@
         <v>2015T3</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>20</v>
       </c>
@@ -1379,7 +1395,7 @@
         <v>2015T4</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>21</v>
       </c>
@@ -1397,7 +1413,7 @@
         <v>2016T1</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>21</v>
       </c>
@@ -1415,7 +1431,7 @@
         <v>2016T2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>21</v>
       </c>
@@ -1433,7 +1449,7 @@
         <v>2016T3</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>21</v>
       </c>
@@ -1451,7 +1467,7 @@
         <v>2016T4</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>22</v>
       </c>
@@ -1469,7 +1485,7 @@
         <v>2017T1</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -1487,7 +1503,7 @@
         <v>2017T2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>22</v>
       </c>
@@ -1505,7 +1521,7 @@
         <v>2017T3</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>22</v>
       </c>
@@ -1523,7 +1539,7 @@
         <v>2017T4</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>23</v>
       </c>
@@ -1541,7 +1557,7 @@
         <v>2018T1</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>23</v>
       </c>
@@ -1559,7 +1575,7 @@
         <v>2018T2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>23</v>
       </c>
@@ -1577,7 +1593,7 @@
         <v>2018T3</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>23</v>
       </c>
@@ -1595,7 +1611,7 @@
         <v>2018T4</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>24</v>
       </c>
@@ -1613,7 +1629,7 @@
         <v>2019T1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -1631,7 +1647,7 @@
         <v>2019T2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>24</v>
       </c>
@@ -1649,7 +1665,7 @@
         <v>2019T3</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>24</v>
       </c>
@@ -1663,11 +1679,11 @@
         <v>241.75364576985601</v>
       </c>
       <c r="E67" t="str">
-        <f t="shared" ref="E67:E83" si="1">_xlfn.CONCAT(A67:B67)</f>
+        <f t="shared" ref="E67:E87" si="1">_xlfn.CONCAT(A67:B67)</f>
         <v>2019T4</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>25</v>
       </c>
@@ -1685,7 +1701,7 @@
         <v>2020T1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>25</v>
       </c>
@@ -1703,7 +1719,7 @@
         <v>2020T2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>25</v>
       </c>
@@ -1721,7 +1737,7 @@
         <v>2020T3</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>25</v>
       </c>
@@ -1739,7 +1755,7 @@
         <v>2020T4</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>26</v>
       </c>
@@ -1757,7 +1773,7 @@
         <v>2021T1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>26</v>
       </c>
@@ -1775,7 +1791,7 @@
         <v>2021T2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>26</v>
       </c>
@@ -1793,7 +1809,7 @@
         <v>2021T3</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>26</v>
       </c>
@@ -1811,7 +1827,7 @@
         <v>2021T4</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>27</v>
       </c>
@@ -1829,7 +1845,7 @@
         <v>2022T1</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>27</v>
       </c>
@@ -1847,7 +1863,7 @@
         <v>2022T2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>27</v>
       </c>
@@ -1865,7 +1881,7 @@
         <v>2022T3</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>27</v>
       </c>
@@ -1883,7 +1899,7 @@
         <v>2022T4</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>28</v>
       </c>
@@ -1901,7 +1917,7 @@
         <v>2023T1</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>28</v>
       </c>
@@ -1919,7 +1935,7 @@
         <v>2023T2</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>28</v>
       </c>
@@ -1937,7 +1953,7 @@
         <v>2023T3</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>28</v>
       </c>
@@ -1955,7 +1971,87 @@
         <v>2023T4</v>
       </c>
     </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>2024</v>
+      </c>
+      <c r="B84" t="s">
+        <v>8</v>
+      </c>
+      <c r="C84" t="s">
+        <v>5</v>
+      </c>
+      <c r="D84">
+        <v>4265.1499999999996</v>
+      </c>
+      <c r="E84" t="str">
+        <f t="shared" si="1"/>
+        <v>2024T1</v>
+      </c>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>2024</v>
+      </c>
+      <c r="B85" t="s">
+        <v>9</v>
+      </c>
+      <c r="C85" t="s">
+        <v>5</v>
+      </c>
+      <c r="D85">
+        <v>5390.54</v>
+      </c>
+      <c r="E85" t="str">
+        <f t="shared" si="1"/>
+        <v>2024T2</v>
+      </c>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>2024</v>
+      </c>
+      <c r="B86" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86">
+        <v>6086.74</v>
+      </c>
+      <c r="E86" t="str">
+        <f t="shared" si="1"/>
+        <v>2024T3</v>
+      </c>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>2024</v>
+      </c>
+      <c r="B87" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87">
+        <v>6643.63</v>
+      </c>
+      <c r="E87" t="str">
+        <f t="shared" si="1"/>
+        <v>2024T4</v>
+      </c>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F88" s="1"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
clases 2 a 5 retoques
</commit_message>
<xml_diff>
--- a/Clase 5 - Markdown, loops y funciones/funciones y loops/bases/ipc_trimestral.xlsx
+++ b/Clase 5 - Markdown, loops y funciones/funciones y loops/bases/ipc_trimestral.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Guido W\curso_aset\Clase 5 - Markdown, loops y funciones\funciones y loops\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AA1763-D1B1-47A3-8D27-0CF2A0F63BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D38BA0-B37E-4138-AE38-067570836DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>